<commit_message>
:up: algumas questoes respondidas - all
</commit_message>
<xml_diff>
--- a/banco_de_dados/historico_respostas.xlsx
+++ b/banco_de_dados/historico_respostas.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -448,6 +448,824 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>15/09/2026 09:22</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>5466</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Engenharia do Trabalho</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>15/09/2026 09:24</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>538</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Gestão da Manutenção e Confiabilidade</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>15/09/2026 09:26</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>5602</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Gestão de Estoques</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>15/09/2026 09:27</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>5601</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Gestão de Estoques</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>15/09/2026 09:27</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>5600</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Gestão de Estoques</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>15/09/2026 09:35</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>5768</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Sustentabilidade</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>15/09/2026 09:38</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>2848</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Contabilidade De Custos</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Custos Diretos E Indiretos</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>15/09/2026 09:41</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>2803</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Contabilidade De Custos</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Apuração Do Custo De Produção</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>15/09/2026 09:41</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2741</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Contabilidade De Custos</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Noções Iniciais Da Contabilidade De Custos</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>15/09/2026 09:51</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>2845</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Contabilidade De Custos</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Custos Diretos E Indiretos</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>15/09/2026 10:23</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>2957</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Contabilidade De Custos</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Tipos de Custeio</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>15/09/2026 10:23</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>2953</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Contabilidade De Custos</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Tipos de Custeio</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>15/09/2026 10:27</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>5065</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Contabilidade Gerencial</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Contabilidade Básica</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>15/09/2026 10:27</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>1412</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Contabilidade Gerencial</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Aspectos Introdutórios</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>15/09/2026 10:27</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2784</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Contabilidade Gerencial</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Contabilidade Básica</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>15/09/2026 10:28</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>1417</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Contabilidade Gerencial</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Contabilidade Básica</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>15/09/2026 10:29</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>1414</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Contabilidade Gerencial</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Aspectos Introdutórios</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>15/09/2026 10:35</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>2783</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Contabilidade Gerencial</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Contabilidade Básica</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>15/09/2026 10:41</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>4777</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Contratação</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Lei Complementar Nº 123 - 2006 e Lei Complementar Nº 155 - 2016</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>15/09/2026 10:41</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>4783</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Contratação</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Lei Complementar Nº 123 - 2006 e Lei Complementar Nº 155 - 2016</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>15/09/2026 10:42</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>4756</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Contratação</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Lei 14.133 - 2021</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>15/09/2026 10:59</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>2548</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Contratação</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Lei nº 14.129 - 2021</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>15/09/2026 10:59</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>4785</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Contratação</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Lei Complementar Nº 123 - 2006 e Lei Complementar Nº 155 - 2016</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>15/09/2026 11:00</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>4780</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Contratação</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Lei Complementar Nº 123 - 2006 e Lei Complementar Nº 155 - 2016</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>15/09/2026 11:01</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>2068</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Estatística</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Probabilidade</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>15/09/2026 11:02</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>2112</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Estatística</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Probabilidade</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>15/09/2026 11:03</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>2098</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Estatística</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Probabilidade</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>15/09/2026 11:07</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>2086</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Estatística</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Probabilidade</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>15/09/2026 11:12</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>2103</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Estatística</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Probabilidade</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>15/09/2026 11:13</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>2596</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Estatística</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Análise Combinatória</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>15/09/2026 11:14</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>1858</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Fundamentos De Engenharia</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Ferramentas Básicas</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
:lady_beetle: consertando algumas questões
</commit_message>
<xml_diff>
--- a/banco_de_dados/historico_respostas.xlsx
+++ b/banco_de_dados/historico_respostas.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1294,6 +1294,32 @@
         <v>1</v>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>15/09/2026 11:29</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>193</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Concordância Verbal e Nominal</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
:up: algumas questoes cadastradas - port
</commit_message>
<xml_diff>
--- a/banco_de_dados/historico_respostas.xlsx
+++ b/banco_de_dados/historico_respostas.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1320,6 +1320,62 @@
         <v>0</v>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>15/09/2026 22:33</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>2676</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Pontuação</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>15/09/2026 22:35</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>2675</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Morfologia</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
:up: algumas questoes respondidas - con esp
</commit_message>
<xml_diff>
--- a/banco_de_dados/historico_respostas.xlsx
+++ b/banco_de_dados/historico_respostas.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F147"/>
+  <dimension ref="A1:F167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1">
@@ -4313,6 +4313,526 @@
         <v>1</v>
       </c>
     </row>
+    <row r="148">
+      <c r="A148" t="n">
+        <v>148</v>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>24/09/2026 10:50</t>
+        </is>
+      </c>
+      <c r="C148" t="n">
+        <v>5260</v>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>Logística</t>
+        </is>
+      </c>
+      <c r="F148" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="n">
+        <v>149</v>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>24/09/2026 10:51</t>
+        </is>
+      </c>
+      <c r="C149" t="n">
+        <v>5429</v>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Gestão da Qualidade</t>
+        </is>
+      </c>
+      <c r="F149" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="n">
+        <v>150</v>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>24/09/2026 10:51</t>
+        </is>
+      </c>
+      <c r="C150" t="n">
+        <v>5776</v>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>Sustentabilidade</t>
+        </is>
+      </c>
+      <c r="F150" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="n">
+        <v>151</v>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>24/09/2026 10:52</t>
+        </is>
+      </c>
+      <c r="C151" t="n">
+        <v>3005</v>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>Gestão da Qualidade</t>
+        </is>
+      </c>
+      <c r="F151" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="n">
+        <v>152</v>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>24/09/2026 10:53</t>
+        </is>
+      </c>
+      <c r="C152" t="n">
+        <v>5137</v>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>Pesquisa Operacional</t>
+        </is>
+      </c>
+      <c r="F152" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="n">
+        <v>153</v>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>24/09/2026 10:56</t>
+        </is>
+      </c>
+      <c r="C153" t="n">
+        <v>823</v>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>Engenharia de Produto</t>
+        </is>
+      </c>
+      <c r="F153" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="n">
+        <v>154</v>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>24/09/2026 10:57</t>
+        </is>
+      </c>
+      <c r="C154" t="n">
+        <v>467</v>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>Pesquisa Operacional</t>
+        </is>
+      </c>
+      <c r="F154" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="n">
+        <v>155</v>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>24/09/2026 10:59</t>
+        </is>
+      </c>
+      <c r="C155" t="n">
+        <v>5590</v>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>Planejamento e Controle da Produção</t>
+        </is>
+      </c>
+      <c r="F155" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="n">
+        <v>156</v>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>24/09/2026 11:01</t>
+        </is>
+      </c>
+      <c r="C156" t="n">
+        <v>5220</v>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>Gestão da Manutenção e Confiabilidade</t>
+        </is>
+      </c>
+      <c r="F156" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="n">
+        <v>157</v>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>24/09/2026 11:02</t>
+        </is>
+      </c>
+      <c r="C157" t="n">
+        <v>5304</v>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>Gestão de Projetos</t>
+        </is>
+      </c>
+      <c r="F157" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="n">
+        <v>158</v>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>24/09/2026 11:02</t>
+        </is>
+      </c>
+      <c r="C158" t="n">
+        <v>5159</v>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>Gestão da Qualidade</t>
+        </is>
+      </c>
+      <c r="F158" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="n">
+        <v>159</v>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>24/09/2026 11:04</t>
+        </is>
+      </c>
+      <c r="C159" t="n">
+        <v>3256</v>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>Processos Decisórios</t>
+        </is>
+      </c>
+      <c r="F159" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="n">
+        <v>160</v>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>24/09/2026 11:05</t>
+        </is>
+      </c>
+      <c r="C160" t="n">
+        <v>5820</v>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>Gestão da Informação</t>
+        </is>
+      </c>
+      <c r="F160" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="n">
+        <v>161</v>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>24/09/2026 11:06</t>
+        </is>
+      </c>
+      <c r="C161" t="n">
+        <v>5178</v>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>Engenharia de Produto</t>
+        </is>
+      </c>
+      <c r="F161" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="n">
+        <v>162</v>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>24/09/2026 11:07</t>
+        </is>
+      </c>
+      <c r="C162" t="n">
+        <v>5761</v>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>Sustentabilidade</t>
+        </is>
+      </c>
+      <c r="F162" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="n">
+        <v>163</v>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>24/09/2026 11:09</t>
+        </is>
+      </c>
+      <c r="C163" t="n">
+        <v>492</v>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>Processos Decisórios</t>
+        </is>
+      </c>
+      <c r="F163" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="n">
+        <v>164</v>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>24/09/2026 11:14</t>
+        </is>
+      </c>
+      <c r="C164" t="n">
+        <v>5128</v>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>Pesquisa Operacional</t>
+        </is>
+      </c>
+      <c r="F164" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="n">
+        <v>165</v>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>24/09/2026 11:15</t>
+        </is>
+      </c>
+      <c r="C165" t="n">
+        <v>710</v>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>Sustentabilidade</t>
+        </is>
+      </c>
+      <c r="F165" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="n">
+        <v>166</v>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>24/09/2026 11:16</t>
+        </is>
+      </c>
+      <c r="C166" t="n">
+        <v>5484</v>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>Engenharia do Trabalho</t>
+        </is>
+      </c>
+      <c r="F166" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="n">
+        <v>167</v>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>24/09/2026 11:17</t>
+        </is>
+      </c>
+      <c r="C167" t="n">
+        <v>5636</v>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>Logística</t>
+        </is>
+      </c>
+      <c r="F167" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
:up: algumas questoes cadastradas - gest econ
</commit_message>
<xml_diff>
--- a/banco_de_dados/historico_respostas.xlsx
+++ b/banco_de_dados/historico_respostas.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F374"/>
+  <dimension ref="A1:F384"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1">
@@ -10287,6 +10287,266 @@
         <v>1</v>
       </c>
     </row>
+    <row r="375">
+      <c r="A375" t="n">
+        <v>375</v>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>27/09/2026 12:43</t>
+        </is>
+      </c>
+      <c r="C375" t="n">
+        <v>5074</v>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>Gestão Econômica</t>
+        </is>
+      </c>
+      <c r="F375" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="n">
+        <v>376</v>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>27/09/2026 12:45</t>
+        </is>
+      </c>
+      <c r="C376" t="n">
+        <v>5067</v>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>Gestão Econômica</t>
+        </is>
+      </c>
+      <c r="F376" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="n">
+        <v>377</v>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>27/09/2026 12:47</t>
+        </is>
+      </c>
+      <c r="C377" t="n">
+        <v>5100</v>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>Gestão Econômica</t>
+        </is>
+      </c>
+      <c r="F377" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="n">
+        <v>378</v>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>27/09/2026 12:48</t>
+        </is>
+      </c>
+      <c r="C378" t="n">
+        <v>5210</v>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>Gestão Econômica</t>
+        </is>
+      </c>
+      <c r="F378" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="n">
+        <v>379</v>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>27/09/2026 12:51</t>
+        </is>
+      </c>
+      <c r="C379" t="n">
+        <v>5215</v>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>Gestão Econômica</t>
+        </is>
+      </c>
+      <c r="F379" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="n">
+        <v>380</v>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>27/09/2026 13:07</t>
+        </is>
+      </c>
+      <c r="C380" t="n">
+        <v>5346</v>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>Gestão Econômica</t>
+        </is>
+      </c>
+      <c r="F380" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="n">
+        <v>381</v>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>27/09/2026 13:14</t>
+        </is>
+      </c>
+      <c r="C381" t="n">
+        <v>5069</v>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>Gestão Econômica</t>
+        </is>
+      </c>
+      <c r="F381" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="n">
+        <v>382</v>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>27/09/2026 13:15</t>
+        </is>
+      </c>
+      <c r="C382" t="n">
+        <v>5075</v>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t>Gestão Econômica</t>
+        </is>
+      </c>
+      <c r="F382" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="n">
+        <v>383</v>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>27/09/2026 13:16</t>
+        </is>
+      </c>
+      <c r="C383" t="n">
+        <v>5211</v>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>Gestão Econômica</t>
+        </is>
+      </c>
+      <c r="F383" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="n">
+        <v>384</v>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>27/09/2026 13:16</t>
+        </is>
+      </c>
+      <c r="C384" t="n">
+        <v>5216</v>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>Gestão Econômica</t>
+        </is>
+      </c>
+      <c r="F384" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
:up: algumas questoes respondidas - estat
</commit_message>
<xml_diff>
--- a/banco_de_dados/historico_respostas.xlsx
+++ b/banco_de_dados/historico_respostas.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F394"/>
+  <dimension ref="A1:F427"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1">
@@ -10811,6 +10811,876 @@
         <v>0</v>
       </c>
     </row>
+    <row r="395">
+      <c r="A395" t="n">
+        <v>395</v>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>27/09/2026 17:29</t>
+        </is>
+      </c>
+      <c r="C395" t="n">
+        <v>1430</v>
+      </c>
+      <c r="D395" t="inlineStr">
+        <is>
+          <t>Contabilidade Gerencial</t>
+        </is>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>Contabilidade Básica</t>
+        </is>
+      </c>
+      <c r="F395" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="n">
+        <v>396</v>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>27/09/2026 17:31</t>
+        </is>
+      </c>
+      <c r="C396" t="n">
+        <v>2782</v>
+      </c>
+      <c r="D396" t="inlineStr">
+        <is>
+          <t>Contabilidade Gerencial</t>
+        </is>
+      </c>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>Contabilidade Básica</t>
+        </is>
+      </c>
+      <c r="F396" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="n">
+        <v>397</v>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>27/09/2026 17:31</t>
+        </is>
+      </c>
+      <c r="C397" t="n">
+        <v>1427</v>
+      </c>
+      <c r="D397" t="inlineStr">
+        <is>
+          <t>Contabilidade Gerencial</t>
+        </is>
+      </c>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t>Contabilidade Básica</t>
+        </is>
+      </c>
+      <c r="F397" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="n">
+        <v>398</v>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>27/09/2026 17:32</t>
+        </is>
+      </c>
+      <c r="C398" t="n">
+        <v>1428</v>
+      </c>
+      <c r="D398" t="inlineStr">
+        <is>
+          <t>Contabilidade Gerencial</t>
+        </is>
+      </c>
+      <c r="E398" t="inlineStr">
+        <is>
+          <t>Contabilidade Básica</t>
+        </is>
+      </c>
+      <c r="F398" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="n">
+        <v>399</v>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>27/09/2026 17:32</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>1426</t>
+        </is>
+      </c>
+      <c r="D399" t="inlineStr">
+        <is>
+          <t>Contabilidade Gerencial</t>
+        </is>
+      </c>
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>Contabilidade Básica</t>
+        </is>
+      </c>
+      <c r="F399" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="n">
+        <v>400</v>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>27/09/2026 17:33</t>
+        </is>
+      </c>
+      <c r="C400" t="n">
+        <v>1418</v>
+      </c>
+      <c r="D400" t="inlineStr">
+        <is>
+          <t>Contabilidade Gerencial</t>
+        </is>
+      </c>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>Contabilidade Básica</t>
+        </is>
+      </c>
+      <c r="F400" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="n">
+        <v>401</v>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>27/09/2026 17:36</t>
+        </is>
+      </c>
+      <c r="C401" t="n">
+        <v>5063</v>
+      </c>
+      <c r="D401" t="inlineStr">
+        <is>
+          <t>Contabilidade Gerencial</t>
+        </is>
+      </c>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>Contabilidade Básica</t>
+        </is>
+      </c>
+      <c r="F401" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="n">
+        <v>402</v>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>27/09/2026 17:37</t>
+        </is>
+      </c>
+      <c r="C402" t="n">
+        <v>1424</v>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t>Contabilidade Gerencial</t>
+        </is>
+      </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>Contabilidade Básica</t>
+        </is>
+      </c>
+      <c r="F402" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="n">
+        <v>403</v>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>27/09/2026 17:38</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>3231</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>Contabilidade Gerencial</t>
+        </is>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>Aspectos Introdutórios</t>
+        </is>
+      </c>
+      <c r="F403" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="n">
+        <v>404</v>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>27/09/2026 17:38</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>3274</t>
+        </is>
+      </c>
+      <c r="D404" t="inlineStr">
+        <is>
+          <t>Contabilidade Gerencial</t>
+        </is>
+      </c>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>Aspectos Introdutórios</t>
+        </is>
+      </c>
+      <c r="F404" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="n">
+        <v>405</v>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>27/09/2026 17:39</t>
+        </is>
+      </c>
+      <c r="C405" t="n">
+        <v>1411</v>
+      </c>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t>Contabilidade Gerencial</t>
+        </is>
+      </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>Aspectos Introdutórios</t>
+        </is>
+      </c>
+      <c r="F405" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="n">
+        <v>406</v>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>27/09/2026 17:41</t>
+        </is>
+      </c>
+      <c r="C406" t="n">
+        <v>5350</v>
+      </c>
+      <c r="D406" t="inlineStr">
+        <is>
+          <t>Contabilidade Gerencial</t>
+        </is>
+      </c>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t>Aspectos Introdutórios</t>
+        </is>
+      </c>
+      <c r="F406" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="n">
+        <v>407</v>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>27/09/2026 17:42</t>
+        </is>
+      </c>
+      <c r="C407" t="n">
+        <v>3200</v>
+      </c>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t>Contabilidade Gerencial</t>
+        </is>
+      </c>
+      <c r="E407" t="inlineStr">
+        <is>
+          <t>Aspectos Introdutórios</t>
+        </is>
+      </c>
+      <c r="F407" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="n">
+        <v>408</v>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>27/09/2026 17:43</t>
+        </is>
+      </c>
+      <c r="C408" t="n">
+        <v>1416</v>
+      </c>
+      <c r="D408" t="inlineStr">
+        <is>
+          <t>Contabilidade Gerencial</t>
+        </is>
+      </c>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>Aspectos Introdutórios</t>
+        </is>
+      </c>
+      <c r="F408" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="n">
+        <v>409</v>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>27/09/2026 17:44</t>
+        </is>
+      </c>
+      <c r="C409" t="n">
+        <v>5205</v>
+      </c>
+      <c r="D409" t="inlineStr">
+        <is>
+          <t>Contabilidade Gerencial</t>
+        </is>
+      </c>
+      <c r="E409" t="inlineStr">
+        <is>
+          <t>Aspectos Introdutórios</t>
+        </is>
+      </c>
+      <c r="F409" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="n">
+        <v>410</v>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>27/09/2026 17:44</t>
+        </is>
+      </c>
+      <c r="C410" t="n">
+        <v>1413</v>
+      </c>
+      <c r="D410" t="inlineStr">
+        <is>
+          <t>Contabilidade Gerencial</t>
+        </is>
+      </c>
+      <c r="E410" t="inlineStr">
+        <is>
+          <t>Aspectos Introdutórios</t>
+        </is>
+      </c>
+      <c r="F410" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="n">
+        <v>411</v>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>27/09/2026 18:00</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>4492</t>
+        </is>
+      </c>
+      <c r="D411" t="inlineStr">
+        <is>
+          <t>Estatística</t>
+        </is>
+      </c>
+      <c r="E411" t="inlineStr">
+        <is>
+          <t>Análise Combinatória</t>
+        </is>
+      </c>
+      <c r="F411" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="n">
+        <v>412</v>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>27/09/2026 18:05</t>
+        </is>
+      </c>
+      <c r="C412" t="n">
+        <v>4508</v>
+      </c>
+      <c r="D412" t="inlineStr">
+        <is>
+          <t>Estatística</t>
+        </is>
+      </c>
+      <c r="E412" t="inlineStr">
+        <is>
+          <t>Análise Combinatória</t>
+        </is>
+      </c>
+      <c r="F412" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="n">
+        <v>413</v>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>27/09/2026 18:09</t>
+        </is>
+      </c>
+      <c r="C413" t="n">
+        <v>2043</v>
+      </c>
+      <c r="D413" t="inlineStr">
+        <is>
+          <t>Estatística</t>
+        </is>
+      </c>
+      <c r="E413" t="inlineStr">
+        <is>
+          <t>Análise Combinatória</t>
+        </is>
+      </c>
+      <c r="F413" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="n">
+        <v>414</v>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>27/09/2026 18:15</t>
+        </is>
+      </c>
+      <c r="C414" t="n">
+        <v>4510</v>
+      </c>
+      <c r="D414" t="inlineStr">
+        <is>
+          <t>Estatística</t>
+        </is>
+      </c>
+      <c r="E414" t="inlineStr">
+        <is>
+          <t>Análise Combinatória</t>
+        </is>
+      </c>
+      <c r="F414" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="n">
+        <v>415</v>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>27/09/2026 18:18</t>
+        </is>
+      </c>
+      <c r="C415" t="n">
+        <v>2060</v>
+      </c>
+      <c r="D415" t="inlineStr">
+        <is>
+          <t>Estatística</t>
+        </is>
+      </c>
+      <c r="E415" t="inlineStr">
+        <is>
+          <t>Análise Combinatória</t>
+        </is>
+      </c>
+      <c r="F415" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="n">
+        <v>416</v>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>27/09/2026 18:22</t>
+        </is>
+      </c>
+      <c r="C416" t="n">
+        <v>2600</v>
+      </c>
+      <c r="D416" t="inlineStr">
+        <is>
+          <t>Estatística</t>
+        </is>
+      </c>
+      <c r="E416" t="inlineStr">
+        <is>
+          <t>Análise Combinatória</t>
+        </is>
+      </c>
+      <c r="F416" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="n">
+        <v>417</v>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>27/09/2026 18:24</t>
+        </is>
+      </c>
+      <c r="C417" t="n">
+        <v>2050</v>
+      </c>
+      <c r="D417" t="inlineStr">
+        <is>
+          <t>Estatística</t>
+        </is>
+      </c>
+      <c r="E417" t="inlineStr">
+        <is>
+          <t>Análise Combinatória</t>
+        </is>
+      </c>
+      <c r="F417" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="n">
+        <v>418</v>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>27/09/2026 18:33</t>
+        </is>
+      </c>
+      <c r="C418" t="n">
+        <v>3404</v>
+      </c>
+      <c r="D418" t="inlineStr">
+        <is>
+          <t>Estatística</t>
+        </is>
+      </c>
+      <c r="E418" t="inlineStr">
+        <is>
+          <t>Análise Combinatória</t>
+        </is>
+      </c>
+      <c r="F418" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="n">
+        <v>419</v>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>27/09/2026 18:38</t>
+        </is>
+      </c>
+      <c r="C419" t="n">
+        <v>4494</v>
+      </c>
+      <c r="D419" t="inlineStr">
+        <is>
+          <t>Estatística</t>
+        </is>
+      </c>
+      <c r="E419" t="inlineStr">
+        <is>
+          <t>Análise Combinatória</t>
+        </is>
+      </c>
+      <c r="F419" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="n">
+        <v>420</v>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>27/09/2026 18:39</t>
+        </is>
+      </c>
+      <c r="C420" t="n">
+        <v>981</v>
+      </c>
+      <c r="D420" t="inlineStr">
+        <is>
+          <t>Estatística</t>
+        </is>
+      </c>
+      <c r="E420" t="inlineStr">
+        <is>
+          <t>Apresentação de Dados</t>
+        </is>
+      </c>
+      <c r="F420" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="n">
+        <v>421</v>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>27/09/2026 18:40</t>
+        </is>
+      </c>
+      <c r="C421" t="n">
+        <v>983</v>
+      </c>
+      <c r="D421" t="inlineStr">
+        <is>
+          <t>Estatística</t>
+        </is>
+      </c>
+      <c r="E421" t="inlineStr">
+        <is>
+          <t>Apresentação de Dados</t>
+        </is>
+      </c>
+      <c r="F421" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="n">
+        <v>422</v>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>27/09/2026 18:46</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>5254</t>
+        </is>
+      </c>
+      <c r="D422" t="inlineStr">
+        <is>
+          <t>Estatística</t>
+        </is>
+      </c>
+      <c r="E422" t="inlineStr">
+        <is>
+          <t>Apresentação de Dados</t>
+        </is>
+      </c>
+      <c r="F422" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="n">
+        <v>423</v>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>27/09/2026 18:46</t>
+        </is>
+      </c>
+      <c r="C423" t="n">
+        <v>982</v>
+      </c>
+      <c r="D423" t="inlineStr">
+        <is>
+          <t>Estatística</t>
+        </is>
+      </c>
+      <c r="E423" t="inlineStr">
+        <is>
+          <t>Apresentação de Dados</t>
+        </is>
+      </c>
+      <c r="F423" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="n">
+        <v>424</v>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>27/09/2026 18:48</t>
+        </is>
+      </c>
+      <c r="C424" t="n">
+        <v>5273</v>
+      </c>
+      <c r="D424" t="inlineStr">
+        <is>
+          <t>Estatística</t>
+        </is>
+      </c>
+      <c r="E424" t="inlineStr">
+        <is>
+          <t>Estimação Pontual e Intervalar</t>
+        </is>
+      </c>
+      <c r="F424" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="n">
+        <v>425</v>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>27/09/2026 18:48</t>
+        </is>
+      </c>
+      <c r="C425" t="n">
+        <v>5298</v>
+      </c>
+      <c r="D425" t="inlineStr">
+        <is>
+          <t>Estatística</t>
+        </is>
+      </c>
+      <c r="E425" t="inlineStr">
+        <is>
+          <t>Estimação Pontual e Intervalar</t>
+        </is>
+      </c>
+      <c r="F425" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="n">
+        <v>426</v>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>27/09/2026 18:49</t>
+        </is>
+      </c>
+      <c r="C426" t="n">
+        <v>5255</v>
+      </c>
+      <c r="D426" t="inlineStr">
+        <is>
+          <t>Estatística</t>
+        </is>
+      </c>
+      <c r="E426" t="inlineStr">
+        <is>
+          <t>Estimação Pontual e Intervalar</t>
+        </is>
+      </c>
+      <c r="F426" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="n">
+        <v>427</v>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>27/09/2026 18:49</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>2764</t>
+        </is>
+      </c>
+      <c r="D427" t="inlineStr">
+        <is>
+          <t>Estatística</t>
+        </is>
+      </c>
+      <c r="E427" t="inlineStr">
+        <is>
+          <t>Estimação Pontual e Intervalar</t>
+        </is>
+      </c>
+      <c r="F427" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
:up: algumas questoes respondidas - cont cust
</commit_message>
<xml_diff>
--- a/banco_de_dados/historico_respostas.xlsx
+++ b/banco_de_dados/historico_respostas.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F534"/>
+  <dimension ref="A1:F541"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="21.44140625" customWidth="1" min="2" max="2"/>
@@ -14478,6 +14478,188 @@
         <v>0</v>
       </c>
     </row>
+    <row r="535">
+      <c r="A535" t="n">
+        <v>536</v>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>28/09/2026 10:18</t>
+        </is>
+      </c>
+      <c r="C535" t="n">
+        <v>2861</v>
+      </c>
+      <c r="D535" t="inlineStr">
+        <is>
+          <t>Contabilidade De Custos</t>
+        </is>
+      </c>
+      <c r="E535" t="inlineStr">
+        <is>
+          <t>Custos Diretos E Indiretos</t>
+        </is>
+      </c>
+      <c r="F535" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="n">
+        <v>537</v>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>28/09/2026 10:20</t>
+        </is>
+      </c>
+      <c r="C536" t="n">
+        <v>6341</v>
+      </c>
+      <c r="D536" t="inlineStr">
+        <is>
+          <t>Contabilidade De Custos</t>
+        </is>
+      </c>
+      <c r="E536" t="inlineStr">
+        <is>
+          <t>Custos Diretos E Indiretos</t>
+        </is>
+      </c>
+      <c r="F536" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="n">
+        <v>538</v>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>28/09/2026 10:29</t>
+        </is>
+      </c>
+      <c r="C537" t="n">
+        <v>2868</v>
+      </c>
+      <c r="D537" t="inlineStr">
+        <is>
+          <t>Contabilidade De Custos</t>
+        </is>
+      </c>
+      <c r="E537" t="inlineStr">
+        <is>
+          <t>Tipos de Custeio</t>
+        </is>
+      </c>
+      <c r="F537" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="n">
+        <v>539</v>
+      </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>29/09/2026 00:24</t>
+        </is>
+      </c>
+      <c r="C538" t="n">
+        <v>2867</v>
+      </c>
+      <c r="D538" t="inlineStr">
+        <is>
+          <t>Contabilidade De Custos</t>
+        </is>
+      </c>
+      <c r="E538" t="inlineStr">
+        <is>
+          <t>Custos Diretos E Indiretos</t>
+        </is>
+      </c>
+      <c r="F538" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="n">
+        <v>540</v>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>29/09/2026 07:16</t>
+        </is>
+      </c>
+      <c r="C539" t="n">
+        <v>2862</v>
+      </c>
+      <c r="D539" t="inlineStr">
+        <is>
+          <t>Contabilidade De Custos</t>
+        </is>
+      </c>
+      <c r="E539" t="inlineStr">
+        <is>
+          <t>Custos Diretos E Indiretos</t>
+        </is>
+      </c>
+      <c r="F539" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="n">
+        <v>541</v>
+      </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>29/09/2026 07:19</t>
+        </is>
+      </c>
+      <c r="C540" t="n">
+        <v>2865</v>
+      </c>
+      <c r="D540" t="inlineStr">
+        <is>
+          <t>Contabilidade De Custos</t>
+        </is>
+      </c>
+      <c r="E540" t="inlineStr">
+        <is>
+          <t>Custos Diretos E Indiretos</t>
+        </is>
+      </c>
+      <c r="F540" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="n">
+        <v>542</v>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>29/09/2026 08:50</t>
+        </is>
+      </c>
+      <c r="C541" t="n">
+        <v>2841</v>
+      </c>
+      <c r="D541" t="inlineStr">
+        <is>
+          <t>Contabilidade De Custos</t>
+        </is>
+      </c>
+      <c r="E541" t="inlineStr">
+        <is>
+          <t>Custos Diretos E Indiretos</t>
+        </is>
+      </c>
+      <c r="F541" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
:up: algumas questoes respondidas - ing
</commit_message>
<xml_diff>
--- a/banco_de_dados/historico_respostas.xlsx
+++ b/banco_de_dados/historico_respostas.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F612"/>
+  <dimension ref="A1:F617"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="21.44140625" customWidth="1" min="2" max="2"/>
@@ -16514,6 +16514,138 @@
         <v>1</v>
       </c>
     </row>
+    <row r="613">
+      <c r="A613" t="n">
+        <v>614</v>
+      </c>
+      <c r="B613" t="inlineStr">
+        <is>
+          <t>29/09/2026 17:37</t>
+        </is>
+      </c>
+      <c r="C613" t="n">
+        <v>970</v>
+      </c>
+      <c r="D613" t="inlineStr">
+        <is>
+          <t>Inglês</t>
+        </is>
+      </c>
+      <c r="E613" t="inlineStr">
+        <is>
+          <t>Vocabulary &amp; Semantics</t>
+        </is>
+      </c>
+      <c r="F613" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" t="n">
+        <v>615</v>
+      </c>
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>29/09/2026 17:38</t>
+        </is>
+      </c>
+      <c r="C614" t="n">
+        <v>969</v>
+      </c>
+      <c r="D614" t="inlineStr">
+        <is>
+          <t>Inglês</t>
+        </is>
+      </c>
+      <c r="E614" t="inlineStr">
+        <is>
+          <t>Vocabulary &amp; Semantics</t>
+        </is>
+      </c>
+      <c r="F614" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" t="n">
+        <v>616</v>
+      </c>
+      <c r="B615" t="inlineStr">
+        <is>
+          <t>29/09/2026 17:38</t>
+        </is>
+      </c>
+      <c r="C615" t="n">
+        <v>968</v>
+      </c>
+      <c r="D615" t="inlineStr">
+        <is>
+          <t>Inglês</t>
+        </is>
+      </c>
+      <c r="E615" t="inlineStr">
+        <is>
+          <t>Vocabulary &amp; Semantics</t>
+        </is>
+      </c>
+      <c r="F615" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" t="n">
+        <v>617</v>
+      </c>
+      <c r="B616" t="inlineStr">
+        <is>
+          <t>29/09/2026 17:39</t>
+        </is>
+      </c>
+      <c r="C616" t="inlineStr">
+        <is>
+          <t>967</t>
+        </is>
+      </c>
+      <c r="D616" t="inlineStr">
+        <is>
+          <t>Inglês</t>
+        </is>
+      </c>
+      <c r="E616" t="inlineStr">
+        <is>
+          <t>Modal Verbs</t>
+        </is>
+      </c>
+      <c r="F616" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" t="n">
+        <v>618</v>
+      </c>
+      <c r="B617" t="inlineStr">
+        <is>
+          <t>29/09/2026 17:40</t>
+        </is>
+      </c>
+      <c r="C617" t="n">
+        <v>966</v>
+      </c>
+      <c r="D617" t="inlineStr">
+        <is>
+          <t>Inglês</t>
+        </is>
+      </c>
+      <c r="E617" t="inlineStr">
+        <is>
+          <t>Reading Comprehension</t>
+        </is>
+      </c>
+      <c r="F617" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
:up: algumas questoes respondidas - contr
</commit_message>
<xml_diff>
--- a/banco_de_dados/historico_respostas.xlsx
+++ b/banco_de_dados/historico_respostas.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F628"/>
+  <dimension ref="A1:F641"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="21.44140625" customWidth="1" min="2" max="2"/>
@@ -16932,6 +16932,344 @@
         <v>1</v>
       </c>
     </row>
+    <row r="629">
+      <c r="A629" t="n">
+        <v>630</v>
+      </c>
+      <c r="B629" t="inlineStr">
+        <is>
+          <t>29/09/2026 18:52</t>
+        </is>
+      </c>
+      <c r="C629" t="n">
+        <v>4846</v>
+      </c>
+      <c r="D629" t="inlineStr">
+        <is>
+          <t>Contratação</t>
+        </is>
+      </c>
+      <c r="E629" t="inlineStr">
+        <is>
+          <t>Lei nº 14.129 - 2021</t>
+        </is>
+      </c>
+      <c r="F629" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" t="n">
+        <v>631</v>
+      </c>
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>29/09/2026 18:54</t>
+        </is>
+      </c>
+      <c r="C630" t="n">
+        <v>2549</v>
+      </c>
+      <c r="D630" t="inlineStr">
+        <is>
+          <t>Contratação</t>
+        </is>
+      </c>
+      <c r="E630" t="inlineStr">
+        <is>
+          <t>Lei nº 14.129 - 2021</t>
+        </is>
+      </c>
+      <c r="F630" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" t="n">
+        <v>632</v>
+      </c>
+      <c r="B631" t="inlineStr">
+        <is>
+          <t>29/09/2026 18:54</t>
+        </is>
+      </c>
+      <c r="C631" t="n">
+        <v>2551</v>
+      </c>
+      <c r="D631" t="inlineStr">
+        <is>
+          <t>Contratação</t>
+        </is>
+      </c>
+      <c r="E631" t="inlineStr">
+        <is>
+          <t>Lei nº 14.129 - 2021</t>
+        </is>
+      </c>
+      <c r="F631" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" t="n">
+        <v>633</v>
+      </c>
+      <c r="B632" t="inlineStr">
+        <is>
+          <t>29/09/2026 18:55</t>
+        </is>
+      </c>
+      <c r="C632" t="n">
+        <v>2557</v>
+      </c>
+      <c r="D632" t="inlineStr">
+        <is>
+          <t>Contratação</t>
+        </is>
+      </c>
+      <c r="E632" t="inlineStr">
+        <is>
+          <t>Lei nº 14.129 - 2021</t>
+        </is>
+      </c>
+      <c r="F632" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" t="n">
+        <v>634</v>
+      </c>
+      <c r="B633" t="inlineStr">
+        <is>
+          <t>29/09/2026 18:56</t>
+        </is>
+      </c>
+      <c r="C633" t="n">
+        <v>2561</v>
+      </c>
+      <c r="D633" t="inlineStr">
+        <is>
+          <t>Contratação</t>
+        </is>
+      </c>
+      <c r="E633" t="inlineStr">
+        <is>
+          <t>Lei nº 14.129 - 2021</t>
+        </is>
+      </c>
+      <c r="F633" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" t="n">
+        <v>635</v>
+      </c>
+      <c r="B634" t="inlineStr">
+        <is>
+          <t>29/09/2026 18:59</t>
+        </is>
+      </c>
+      <c r="C634" t="n">
+        <v>4857</v>
+      </c>
+      <c r="D634" t="inlineStr">
+        <is>
+          <t>Contratação</t>
+        </is>
+      </c>
+      <c r="E634" t="inlineStr">
+        <is>
+          <t>Lei nº 14.129 - 2021</t>
+        </is>
+      </c>
+      <c r="F634" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" t="n">
+        <v>636</v>
+      </c>
+      <c r="B635" t="inlineStr">
+        <is>
+          <t>29/09/2026 19:00</t>
+        </is>
+      </c>
+      <c r="C635" t="n">
+        <v>2520</v>
+      </c>
+      <c r="D635" t="inlineStr">
+        <is>
+          <t>Contratação</t>
+        </is>
+      </c>
+      <c r="E635" t="inlineStr">
+        <is>
+          <t>Lei nº 14.129 - 2021</t>
+        </is>
+      </c>
+      <c r="F635" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" t="n">
+        <v>637</v>
+      </c>
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>29/09/2026 19:01</t>
+        </is>
+      </c>
+      <c r="C636" t="n">
+        <v>4862</v>
+      </c>
+      <c r="D636" t="inlineStr">
+        <is>
+          <t>Contratação</t>
+        </is>
+      </c>
+      <c r="E636" t="inlineStr">
+        <is>
+          <t>Lei Complementar Nº 123 - 2006 e Lei Complementar Nº 155 - 2016</t>
+        </is>
+      </c>
+      <c r="F636" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="n">
+        <v>638</v>
+      </c>
+      <c r="B637" t="inlineStr">
+        <is>
+          <t>29/09/2026 19:02</t>
+        </is>
+      </c>
+      <c r="C637" t="n">
+        <v>4827</v>
+      </c>
+      <c r="D637" t="inlineStr">
+        <is>
+          <t>Contratação</t>
+        </is>
+      </c>
+      <c r="E637" t="inlineStr">
+        <is>
+          <t>Lei Complementar Nº 123 - 2006 e Lei Complementar Nº 155 - 2016</t>
+        </is>
+      </c>
+      <c r="F637" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" t="n">
+        <v>639</v>
+      </c>
+      <c r="B638" t="inlineStr">
+        <is>
+          <t>29/09/2026 19:03</t>
+        </is>
+      </c>
+      <c r="C638" t="n">
+        <v>4863</v>
+      </c>
+      <c r="D638" t="inlineStr">
+        <is>
+          <t>Contratação</t>
+        </is>
+      </c>
+      <c r="E638" t="inlineStr">
+        <is>
+          <t>Lei Complementar Nº 123 - 2006 e Lei Complementar Nº 155 - 2016</t>
+        </is>
+      </c>
+      <c r="F638" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" t="n">
+        <v>640</v>
+      </c>
+      <c r="B639" t="inlineStr">
+        <is>
+          <t>29/09/2026 19:04</t>
+        </is>
+      </c>
+      <c r="C639" t="n">
+        <v>4868</v>
+      </c>
+      <c r="D639" t="inlineStr">
+        <is>
+          <t>Contratação</t>
+        </is>
+      </c>
+      <c r="E639" t="inlineStr">
+        <is>
+          <t>Lei Complementar Nº 123 - 2006 e Lei Complementar Nº 155 - 2016</t>
+        </is>
+      </c>
+      <c r="F639" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" t="n">
+        <v>641</v>
+      </c>
+      <c r="B640" t="inlineStr">
+        <is>
+          <t>29/09/2026 19:05</t>
+        </is>
+      </c>
+      <c r="C640" t="n">
+        <v>4860</v>
+      </c>
+      <c r="D640" t="inlineStr">
+        <is>
+          <t>Contratação</t>
+        </is>
+      </c>
+      <c r="E640" t="inlineStr">
+        <is>
+          <t>Lei Complementar Nº 123 - 2006 e Lei Complementar Nº 155 - 2016</t>
+        </is>
+      </c>
+      <c r="F640" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" t="n">
+        <v>642</v>
+      </c>
+      <c r="B641" t="inlineStr">
+        <is>
+          <t>29/09/2026 19:06</t>
+        </is>
+      </c>
+      <c r="C641" t="n">
+        <v>4788</v>
+      </c>
+      <c r="D641" t="inlineStr">
+        <is>
+          <t>Contratação</t>
+        </is>
+      </c>
+      <c r="E641" t="inlineStr">
+        <is>
+          <t>Lei Complementar Nº 123 - 2006 e Lei Complementar Nº 155 - 2016</t>
+        </is>
+      </c>
+      <c r="F641" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
:up: algumas questoes respondidas - mat fin
</commit_message>
<xml_diff>
--- a/banco_de_dados/historico_respostas.xlsx
+++ b/banco_de_dados/historico_respostas.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F690"/>
+  <dimension ref="A1:F691"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="21.44140625" customWidth="1" min="2" max="2"/>
@@ -18548,6 +18548,32 @@
         <v>1</v>
       </c>
     </row>
+    <row r="691">
+      <c r="A691" t="n">
+        <v>692</v>
+      </c>
+      <c r="B691" t="inlineStr">
+        <is>
+          <t>29/09/2026 22:50</t>
+        </is>
+      </c>
+      <c r="C691" t="n">
+        <v>1283</v>
+      </c>
+      <c r="D691" t="inlineStr">
+        <is>
+          <t>Matemática Financeira</t>
+        </is>
+      </c>
+      <c r="E691" t="inlineStr">
+        <is>
+          <t>Juros Compostos</t>
+        </is>
+      </c>
+      <c r="F691" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
:checkered_flag: plano para a primeira semana montado
</commit_message>
<xml_diff>
--- a/banco_de_dados/historico_respostas.xlsx
+++ b/banco_de_dados/historico_respostas.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F691"/>
+  <dimension ref="A1:F720"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="21.44140625" customWidth="1" min="2" max="2"/>
@@ -18574,6 +18574,760 @@
         <v>1</v>
       </c>
     </row>
+    <row r="692">
+      <c r="A692" t="n">
+        <v>693</v>
+      </c>
+      <c r="B692" t="inlineStr">
+        <is>
+          <t>29/09/2026 23:05</t>
+        </is>
+      </c>
+      <c r="C692" t="n">
+        <v>1256</v>
+      </c>
+      <c r="D692" t="inlineStr">
+        <is>
+          <t>Matemática Financeira</t>
+        </is>
+      </c>
+      <c r="E692" t="inlineStr">
+        <is>
+          <t>Juros Simples</t>
+        </is>
+      </c>
+      <c r="F692" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" t="n">
+        <v>694</v>
+      </c>
+      <c r="B693" t="inlineStr">
+        <is>
+          <t>29/09/2026 23:09</t>
+        </is>
+      </c>
+      <c r="C693" t="n">
+        <v>1259</v>
+      </c>
+      <c r="D693" t="inlineStr">
+        <is>
+          <t>Matemática Financeira</t>
+        </is>
+      </c>
+      <c r="E693" t="inlineStr">
+        <is>
+          <t>Juros Simples</t>
+        </is>
+      </c>
+      <c r="F693" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" t="n">
+        <v>695</v>
+      </c>
+      <c r="B694" t="inlineStr">
+        <is>
+          <t>29/09/2026 23:13</t>
+        </is>
+      </c>
+      <c r="C694" t="n">
+        <v>1247</v>
+      </c>
+      <c r="D694" t="inlineStr">
+        <is>
+          <t>Matemática Financeira</t>
+        </is>
+      </c>
+      <c r="E694" t="inlineStr">
+        <is>
+          <t>Juros Simples</t>
+        </is>
+      </c>
+      <c r="F694" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" t="n">
+        <v>696</v>
+      </c>
+      <c r="B695" t="inlineStr">
+        <is>
+          <t>29/09/2026 23:18</t>
+        </is>
+      </c>
+      <c r="C695" t="n">
+        <v>1252</v>
+      </c>
+      <c r="D695" t="inlineStr">
+        <is>
+          <t>Matemática Financeira</t>
+        </is>
+      </c>
+      <c r="E695" t="inlineStr">
+        <is>
+          <t>Juros Simples</t>
+        </is>
+      </c>
+      <c r="F695" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" t="n">
+        <v>697</v>
+      </c>
+      <c r="B696" t="inlineStr">
+        <is>
+          <t>29/09/2026 23:21</t>
+        </is>
+      </c>
+      <c r="C696" t="n">
+        <v>1253</v>
+      </c>
+      <c r="D696" t="inlineStr">
+        <is>
+          <t>Matemática Financeira</t>
+        </is>
+      </c>
+      <c r="E696" t="inlineStr">
+        <is>
+          <t>Juros Simples</t>
+        </is>
+      </c>
+      <c r="F696" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" t="n">
+        <v>698</v>
+      </c>
+      <c r="B697" t="inlineStr">
+        <is>
+          <t>29/09/2026 23:37</t>
+        </is>
+      </c>
+      <c r="C697" t="n">
+        <v>1246</v>
+      </c>
+      <c r="D697" t="inlineStr">
+        <is>
+          <t>Matemática Financeira</t>
+        </is>
+      </c>
+      <c r="E697" t="inlineStr">
+        <is>
+          <t>Juros Simples</t>
+        </is>
+      </c>
+      <c r="F697" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" t="n">
+        <v>699</v>
+      </c>
+      <c r="B698" t="inlineStr">
+        <is>
+          <t>30/09/2026 08:04</t>
+        </is>
+      </c>
+      <c r="C698" t="n">
+        <v>1257</v>
+      </c>
+      <c r="D698" t="inlineStr">
+        <is>
+          <t>Matemática Financeira</t>
+        </is>
+      </c>
+      <c r="E698" t="inlineStr">
+        <is>
+          <t>Juros Simples</t>
+        </is>
+      </c>
+      <c r="F698" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" t="n">
+        <v>700</v>
+      </c>
+      <c r="B699" t="inlineStr">
+        <is>
+          <t>30/09/2026 08:06</t>
+        </is>
+      </c>
+      <c r="C699" t="n">
+        <v>5313</v>
+      </c>
+      <c r="D699" t="inlineStr">
+        <is>
+          <t>Matemática Financeira</t>
+        </is>
+      </c>
+      <c r="E699" t="inlineStr">
+        <is>
+          <t>Juros Simples</t>
+        </is>
+      </c>
+      <c r="F699" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" t="n">
+        <v>701</v>
+      </c>
+      <c r="B700" t="inlineStr">
+        <is>
+          <t>30/09/2026 08:28</t>
+        </is>
+      </c>
+      <c r="C700" t="n">
+        <v>1254</v>
+      </c>
+      <c r="D700" t="inlineStr">
+        <is>
+          <t>Matemática Financeira</t>
+        </is>
+      </c>
+      <c r="E700" t="inlineStr">
+        <is>
+          <t>Juros Simples</t>
+        </is>
+      </c>
+      <c r="F700" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" t="n">
+        <v>702</v>
+      </c>
+      <c r="B701" t="inlineStr">
+        <is>
+          <t>30/09/2026 08:29</t>
+        </is>
+      </c>
+      <c r="C701" t="n">
+        <v>1244</v>
+      </c>
+      <c r="D701" t="inlineStr">
+        <is>
+          <t>Matemática Financeira</t>
+        </is>
+      </c>
+      <c r="E701" t="inlineStr">
+        <is>
+          <t>Juros Simples</t>
+        </is>
+      </c>
+      <c r="F701" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" t="n">
+        <v>703</v>
+      </c>
+      <c r="B702" t="inlineStr">
+        <is>
+          <t>30/09/2026 08:33</t>
+        </is>
+      </c>
+      <c r="C702" t="n">
+        <v>5312</v>
+      </c>
+      <c r="D702" t="inlineStr">
+        <is>
+          <t>Matemática Financeira</t>
+        </is>
+      </c>
+      <c r="E702" t="inlineStr">
+        <is>
+          <t>Operações de Desconto</t>
+        </is>
+      </c>
+      <c r="F702" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" t="n">
+        <v>704</v>
+      </c>
+      <c r="B703" t="inlineStr">
+        <is>
+          <t>30/09/2026 08:33</t>
+        </is>
+      </c>
+      <c r="C703" t="n">
+        <v>3094</v>
+      </c>
+      <c r="D703" t="inlineStr">
+        <is>
+          <t>Matemática Financeira</t>
+        </is>
+      </c>
+      <c r="E703" t="inlineStr">
+        <is>
+          <t>Operações de Desconto</t>
+        </is>
+      </c>
+      <c r="F703" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" t="n">
+        <v>705</v>
+      </c>
+      <c r="B704" t="inlineStr">
+        <is>
+          <t>30/09/2026 08:33</t>
+        </is>
+      </c>
+      <c r="C704" t="n">
+        <v>3089</v>
+      </c>
+      <c r="D704" t="inlineStr">
+        <is>
+          <t>Matemática Financeira</t>
+        </is>
+      </c>
+      <c r="E704" t="inlineStr">
+        <is>
+          <t>Operações de Desconto</t>
+        </is>
+      </c>
+      <c r="F704" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" t="n">
+        <v>706</v>
+      </c>
+      <c r="B705" t="inlineStr">
+        <is>
+          <t>30/09/2026 08:33</t>
+        </is>
+      </c>
+      <c r="C705" t="n">
+        <v>3092</v>
+      </c>
+      <c r="D705" t="inlineStr">
+        <is>
+          <t>Matemática Financeira</t>
+        </is>
+      </c>
+      <c r="E705" t="inlineStr">
+        <is>
+          <t>Operações de Desconto</t>
+        </is>
+      </c>
+      <c r="F705" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" t="n">
+        <v>707</v>
+      </c>
+      <c r="B706" t="inlineStr">
+        <is>
+          <t>30/09/2026 08:33</t>
+        </is>
+      </c>
+      <c r="C706" t="n">
+        <v>3095</v>
+      </c>
+      <c r="D706" t="inlineStr">
+        <is>
+          <t>Matemática Financeira</t>
+        </is>
+      </c>
+      <c r="E706" t="inlineStr">
+        <is>
+          <t>Operações de Desconto</t>
+        </is>
+      </c>
+      <c r="F706" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" t="n">
+        <v>708</v>
+      </c>
+      <c r="B707" t="inlineStr">
+        <is>
+          <t>30/09/2026 08:34</t>
+        </is>
+      </c>
+      <c r="C707" t="n">
+        <v>3085</v>
+      </c>
+      <c r="D707" t="inlineStr">
+        <is>
+          <t>Matemática Financeira</t>
+        </is>
+      </c>
+      <c r="E707" t="inlineStr">
+        <is>
+          <t>Operações de Desconto</t>
+        </is>
+      </c>
+      <c r="F707" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" t="n">
+        <v>709</v>
+      </c>
+      <c r="B708" t="inlineStr">
+        <is>
+          <t>30/09/2026 08:34</t>
+        </is>
+      </c>
+      <c r="C708" t="n">
+        <v>3090</v>
+      </c>
+      <c r="D708" t="inlineStr">
+        <is>
+          <t>Matemática Financeira</t>
+        </is>
+      </c>
+      <c r="E708" t="inlineStr">
+        <is>
+          <t>Operações de Desconto</t>
+        </is>
+      </c>
+      <c r="F708" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" t="n">
+        <v>710</v>
+      </c>
+      <c r="B709" t="inlineStr">
+        <is>
+          <t>30/09/2026 08:34</t>
+        </is>
+      </c>
+      <c r="C709" t="n">
+        <v>3083</v>
+      </c>
+      <c r="D709" t="inlineStr">
+        <is>
+          <t>Matemática Financeira</t>
+        </is>
+      </c>
+      <c r="E709" t="inlineStr">
+        <is>
+          <t>Operações de Desconto</t>
+        </is>
+      </c>
+      <c r="F709" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" t="n">
+        <v>711</v>
+      </c>
+      <c r="B710" t="inlineStr">
+        <is>
+          <t>30/09/2026 08:34</t>
+        </is>
+      </c>
+      <c r="C710" t="n">
+        <v>3084</v>
+      </c>
+      <c r="D710" t="inlineStr">
+        <is>
+          <t>Matemática Financeira</t>
+        </is>
+      </c>
+      <c r="E710" t="inlineStr">
+        <is>
+          <t>Operações de Desconto</t>
+        </is>
+      </c>
+      <c r="F710" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" t="n">
+        <v>712</v>
+      </c>
+      <c r="B711" t="inlineStr">
+        <is>
+          <t>30/09/2026 08:34</t>
+        </is>
+      </c>
+      <c r="C711" t="n">
+        <v>3093</v>
+      </c>
+      <c r="D711" t="inlineStr">
+        <is>
+          <t>Matemática Financeira</t>
+        </is>
+      </c>
+      <c r="E711" t="inlineStr">
+        <is>
+          <t>Operações de Desconto</t>
+        </is>
+      </c>
+      <c r="F711" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" t="n">
+        <v>713</v>
+      </c>
+      <c r="B712" t="inlineStr">
+        <is>
+          <t>30/09/2026 08:41</t>
+        </is>
+      </c>
+      <c r="C712" t="n">
+        <v>3098</v>
+      </c>
+      <c r="D712" t="inlineStr">
+        <is>
+          <t>Matemática Financeira</t>
+        </is>
+      </c>
+      <c r="E712" t="inlineStr">
+        <is>
+          <t>Taxas</t>
+        </is>
+      </c>
+      <c r="F712" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" t="n">
+        <v>714</v>
+      </c>
+      <c r="B713" t="inlineStr">
+        <is>
+          <t>30/09/2026 08:51</t>
+        </is>
+      </c>
+      <c r="C713" t="n">
+        <v>5314</v>
+      </c>
+      <c r="D713" t="inlineStr">
+        <is>
+          <t>Matemática Financeira</t>
+        </is>
+      </c>
+      <c r="E713" t="inlineStr">
+        <is>
+          <t>Taxas</t>
+        </is>
+      </c>
+      <c r="F713" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" t="n">
+        <v>715</v>
+      </c>
+      <c r="B714" t="inlineStr">
+        <is>
+          <t>30/09/2026 08:51</t>
+        </is>
+      </c>
+      <c r="C714" t="n">
+        <v>3097</v>
+      </c>
+      <c r="D714" t="inlineStr">
+        <is>
+          <t>Matemática Financeira</t>
+        </is>
+      </c>
+      <c r="E714" t="inlineStr">
+        <is>
+          <t>Taxas</t>
+        </is>
+      </c>
+      <c r="F714" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" t="n">
+        <v>716</v>
+      </c>
+      <c r="B715" t="inlineStr">
+        <is>
+          <t>30/09/2026 08:51</t>
+        </is>
+      </c>
+      <c r="C715" t="n">
+        <v>5322</v>
+      </c>
+      <c r="D715" t="inlineStr">
+        <is>
+          <t>Matemática Financeira</t>
+        </is>
+      </c>
+      <c r="E715" t="inlineStr">
+        <is>
+          <t>Taxas</t>
+        </is>
+      </c>
+      <c r="F715" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" t="n">
+        <v>717</v>
+      </c>
+      <c r="B716" t="inlineStr">
+        <is>
+          <t>30/09/2026 08:51</t>
+        </is>
+      </c>
+      <c r="C716" t="n">
+        <v>3099</v>
+      </c>
+      <c r="D716" t="inlineStr">
+        <is>
+          <t>Matemática Financeira</t>
+        </is>
+      </c>
+      <c r="E716" t="inlineStr">
+        <is>
+          <t>Taxas</t>
+        </is>
+      </c>
+      <c r="F716" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" t="n">
+        <v>718</v>
+      </c>
+      <c r="B717" t="inlineStr">
+        <is>
+          <t>30/09/2026 08:51</t>
+        </is>
+      </c>
+      <c r="C717" t="n">
+        <v>3232</v>
+      </c>
+      <c r="D717" t="inlineStr">
+        <is>
+          <t>Matemática Financeira</t>
+        </is>
+      </c>
+      <c r="E717" t="inlineStr">
+        <is>
+          <t>Taxas</t>
+        </is>
+      </c>
+      <c r="F717" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" t="n">
+        <v>719</v>
+      </c>
+      <c r="B718" t="inlineStr">
+        <is>
+          <t>30/09/2026 08:51</t>
+        </is>
+      </c>
+      <c r="C718" t="n">
+        <v>3100</v>
+      </c>
+      <c r="D718" t="inlineStr">
+        <is>
+          <t>Matemática Financeira</t>
+        </is>
+      </c>
+      <c r="E718" t="inlineStr">
+        <is>
+          <t>Taxas</t>
+        </is>
+      </c>
+      <c r="F718" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" t="n">
+        <v>720</v>
+      </c>
+      <c r="B719" t="inlineStr">
+        <is>
+          <t>30/09/2026 08:52</t>
+        </is>
+      </c>
+      <c r="C719" t="n">
+        <v>3102</v>
+      </c>
+      <c r="D719" t="inlineStr">
+        <is>
+          <t>Matemática Financeira</t>
+        </is>
+      </c>
+      <c r="E719" t="inlineStr">
+        <is>
+          <t>Taxas</t>
+        </is>
+      </c>
+      <c r="F719" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" t="n">
+        <v>721</v>
+      </c>
+      <c r="B720" t="inlineStr">
+        <is>
+          <t>30/09/2026 08:52</t>
+        </is>
+      </c>
+      <c r="C720" t="n">
+        <v>3096</v>
+      </c>
+      <c r="D720" t="inlineStr">
+        <is>
+          <t>Matemática Financeira</t>
+        </is>
+      </c>
+      <c r="E720" t="inlineStr">
+        <is>
+          <t>Taxas</t>
+        </is>
+      </c>
+      <c r="F720" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
:up: simulado geral respondido
</commit_message>
<xml_diff>
--- a/banco_de_dados/historico_respostas.xlsx
+++ b/banco_de_dados/historico_respostas.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F735"/>
+  <dimension ref="A1:F806"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="21.44140625" customWidth="1" min="2" max="2"/>
@@ -19724,6 +19724,1870 @@
         <v>0</v>
       </c>
     </row>
+    <row r="736">
+      <c r="A736" t="n">
+        <v>737</v>
+      </c>
+      <c r="B736" t="inlineStr">
+        <is>
+          <t>11/10/2026 08:00</t>
+        </is>
+      </c>
+      <c r="C736" t="n">
+        <v>5335</v>
+      </c>
+      <c r="D736" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E736" t="inlineStr">
+        <is>
+          <t>Gestão de Estoques</t>
+        </is>
+      </c>
+      <c r="F736" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" t="n">
+        <v>738</v>
+      </c>
+      <c r="B737" t="inlineStr">
+        <is>
+          <t>11/10/2026 08:01</t>
+        </is>
+      </c>
+      <c r="C737" t="n">
+        <v>5025</v>
+      </c>
+      <c r="D737" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E737" t="inlineStr">
+        <is>
+          <t>Gestão da Qualidade</t>
+        </is>
+      </c>
+      <c r="F737" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" t="n">
+        <v>739</v>
+      </c>
+      <c r="B738" t="inlineStr">
+        <is>
+          <t>11/10/2026 08:03</t>
+        </is>
+      </c>
+      <c r="C738" t="n">
+        <v>5098</v>
+      </c>
+      <c r="D738" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E738" t="inlineStr">
+        <is>
+          <t>Gestão da Qualidade</t>
+        </is>
+      </c>
+      <c r="F738" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" t="n">
+        <v>740</v>
+      </c>
+      <c r="B739" t="inlineStr">
+        <is>
+          <t>11/10/2026 08:04</t>
+        </is>
+      </c>
+      <c r="C739" t="n">
+        <v>3041</v>
+      </c>
+      <c r="D739" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E739" t="inlineStr">
+        <is>
+          <t>Gestão da Tecnologia</t>
+        </is>
+      </c>
+      <c r="F739" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" t="n">
+        <v>741</v>
+      </c>
+      <c r="B740" t="inlineStr">
+        <is>
+          <t>11/10/2026 08:07</t>
+        </is>
+      </c>
+      <c r="C740" t="n">
+        <v>5646</v>
+      </c>
+      <c r="D740" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E740" t="inlineStr">
+        <is>
+          <t>Gestão da Cadeia de Suprimentos</t>
+        </is>
+      </c>
+      <c r="F740" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" t="n">
+        <v>742</v>
+      </c>
+      <c r="B741" t="inlineStr">
+        <is>
+          <t>11/10/2026 08:08</t>
+        </is>
+      </c>
+      <c r="C741" t="n">
+        <v>762</v>
+      </c>
+      <c r="D741" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E741" t="inlineStr">
+        <is>
+          <t>Engenharia Organizacional</t>
+        </is>
+      </c>
+      <c r="F741" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" t="n">
+        <v>743</v>
+      </c>
+      <c r="B742" t="inlineStr">
+        <is>
+          <t>11/10/2026 08:11</t>
+        </is>
+      </c>
+      <c r="C742" t="n">
+        <v>5487</v>
+      </c>
+      <c r="D742" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E742" t="inlineStr">
+        <is>
+          <t>Engenharia do Trabalho</t>
+        </is>
+      </c>
+      <c r="F742" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" t="n">
+        <v>744</v>
+      </c>
+      <c r="B743" t="inlineStr">
+        <is>
+          <t>11/10/2026 08:12</t>
+        </is>
+      </c>
+      <c r="C743" t="n">
+        <v>2655</v>
+      </c>
+      <c r="D743" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E743" t="inlineStr">
+        <is>
+          <t>Gestão da Tecnologia</t>
+        </is>
+      </c>
+      <c r="F743" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" t="n">
+        <v>745</v>
+      </c>
+      <c r="B744" t="inlineStr">
+        <is>
+          <t>11/10/2026 08:13</t>
+        </is>
+      </c>
+      <c r="C744" t="n">
+        <v>2722</v>
+      </c>
+      <c r="D744" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E744" t="inlineStr">
+        <is>
+          <t>Gestão de Projetos</t>
+        </is>
+      </c>
+      <c r="F744" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" t="n">
+        <v>746</v>
+      </c>
+      <c r="B745" t="inlineStr">
+        <is>
+          <t>11/10/2026 08:15</t>
+        </is>
+      </c>
+      <c r="C745" t="n">
+        <v>5817</v>
+      </c>
+      <c r="D745" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E745" t="inlineStr">
+        <is>
+          <t>Planejamento e Controle da Produção</t>
+        </is>
+      </c>
+      <c r="F745" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" t="n">
+        <v>747</v>
+      </c>
+      <c r="B746" t="inlineStr">
+        <is>
+          <t>11/10/2026 08:16</t>
+        </is>
+      </c>
+      <c r="C746" t="n">
+        <v>3319</v>
+      </c>
+      <c r="D746" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E746" t="inlineStr">
+        <is>
+          <t>Gestão da Qualidade</t>
+        </is>
+      </c>
+      <c r="F746" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" t="n">
+        <v>748</v>
+      </c>
+      <c r="B747" t="inlineStr">
+        <is>
+          <t>11/10/2026 08:17</t>
+        </is>
+      </c>
+      <c r="C747" t="n">
+        <v>5718</v>
+      </c>
+      <c r="D747" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E747" t="inlineStr">
+        <is>
+          <t>Sustentabilidade</t>
+        </is>
+      </c>
+      <c r="F747" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" t="n">
+        <v>749</v>
+      </c>
+      <c r="B748" t="inlineStr">
+        <is>
+          <t>11/10/2026 08:18</t>
+        </is>
+      </c>
+      <c r="C748" t="inlineStr">
+        <is>
+          <t>2637</t>
+        </is>
+      </c>
+      <c r="D748" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E748" t="inlineStr">
+        <is>
+          <t>Gestão da Tecnologia</t>
+        </is>
+      </c>
+      <c r="F748" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" t="n">
+        <v>750</v>
+      </c>
+      <c r="B749" t="inlineStr">
+        <is>
+          <t>11/10/2026 08:19</t>
+        </is>
+      </c>
+      <c r="C749" t="inlineStr">
+        <is>
+          <t>5569</t>
+        </is>
+      </c>
+      <c r="D749" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E749" t="inlineStr">
+        <is>
+          <t>Gestão da Cadeia de Suprimentos</t>
+        </is>
+      </c>
+      <c r="F749" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" t="n">
+        <v>751</v>
+      </c>
+      <c r="B750" t="inlineStr">
+        <is>
+          <t>11/10/2026 08:21</t>
+        </is>
+      </c>
+      <c r="C750" t="n">
+        <v>681</v>
+      </c>
+      <c r="D750" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E750" t="inlineStr">
+        <is>
+          <t>Engenharia do Trabalho</t>
+        </is>
+      </c>
+      <c r="F750" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" t="n">
+        <v>752</v>
+      </c>
+      <c r="B751" t="inlineStr">
+        <is>
+          <t>11/10/2026 08:22</t>
+        </is>
+      </c>
+      <c r="C751" t="n">
+        <v>2725</v>
+      </c>
+      <c r="D751" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E751" t="inlineStr">
+        <is>
+          <t>Gestão de Projetos</t>
+        </is>
+      </c>
+      <c r="F751" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" t="n">
+        <v>753</v>
+      </c>
+      <c r="B752" t="inlineStr">
+        <is>
+          <t>11/10/2026 08:23</t>
+        </is>
+      </c>
+      <c r="C752" t="inlineStr">
+        <is>
+          <t>499</t>
+        </is>
+      </c>
+      <c r="D752" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E752" t="inlineStr">
+        <is>
+          <t>Engenharia Organizacional</t>
+        </is>
+      </c>
+      <c r="F752" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" t="n">
+        <v>754</v>
+      </c>
+      <c r="B753" t="inlineStr">
+        <is>
+          <t>11/10/2026 08:23</t>
+        </is>
+      </c>
+      <c r="C753" t="inlineStr">
+        <is>
+          <t>5659</t>
+        </is>
+      </c>
+      <c r="D753" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E753" t="inlineStr">
+        <is>
+          <t>Logística</t>
+        </is>
+      </c>
+      <c r="F753" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" t="n">
+        <v>755</v>
+      </c>
+      <c r="B754" t="inlineStr">
+        <is>
+          <t>11/10/2026 08:25</t>
+        </is>
+      </c>
+      <c r="C754" t="n">
+        <v>4959</v>
+      </c>
+      <c r="D754" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E754" t="inlineStr">
+        <is>
+          <t>Gestão da Cadeia de Suprimentos</t>
+        </is>
+      </c>
+      <c r="F754" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" t="n">
+        <v>756</v>
+      </c>
+      <c r="B755" t="inlineStr">
+        <is>
+          <t>11/10/2026 08:25</t>
+        </is>
+      </c>
+      <c r="C755" t="n">
+        <v>5607</v>
+      </c>
+      <c r="D755" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E755" t="inlineStr">
+        <is>
+          <t>Logística</t>
+        </is>
+      </c>
+      <c r="F755" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="756">
+      <c r="A756" t="n">
+        <v>757</v>
+      </c>
+      <c r="B756" t="inlineStr">
+        <is>
+          <t>11/10/2026 08:26</t>
+        </is>
+      </c>
+      <c r="C756" t="n">
+        <v>632</v>
+      </c>
+      <c r="D756" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E756" t="inlineStr">
+        <is>
+          <t>Engenharia de Produto</t>
+        </is>
+      </c>
+      <c r="F756" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" t="n">
+        <v>758</v>
+      </c>
+      <c r="B757" t="inlineStr">
+        <is>
+          <t>11/10/2026 08:29</t>
+        </is>
+      </c>
+      <c r="C757" t="n">
+        <v>817</v>
+      </c>
+      <c r="D757" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E757" t="inlineStr">
+        <is>
+          <t>Gestão da Qualidade</t>
+        </is>
+      </c>
+      <c r="F757" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="758">
+      <c r="A758" t="n">
+        <v>759</v>
+      </c>
+      <c r="B758" t="inlineStr">
+        <is>
+          <t>11/10/2026 08:30</t>
+        </is>
+      </c>
+      <c r="C758" t="n">
+        <v>866</v>
+      </c>
+      <c r="D758" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E758" t="inlineStr">
+        <is>
+          <t>Engenharia Organizacional</t>
+        </is>
+      </c>
+      <c r="F758" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" t="n">
+        <v>760</v>
+      </c>
+      <c r="B759" t="inlineStr">
+        <is>
+          <t>11/10/2026 08:32</t>
+        </is>
+      </c>
+      <c r="C759" t="n">
+        <v>5447</v>
+      </c>
+      <c r="D759" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E759" t="inlineStr">
+        <is>
+          <t>Engenharia do Trabalho</t>
+        </is>
+      </c>
+      <c r="F759" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="760">
+      <c r="A760" t="n">
+        <v>761</v>
+      </c>
+      <c r="B760" t="inlineStr">
+        <is>
+          <t>11/10/2026 08:32</t>
+        </is>
+      </c>
+      <c r="C760" t="n">
+        <v>636</v>
+      </c>
+      <c r="D760" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E760" t="inlineStr">
+        <is>
+          <t>Engenharia de Produto</t>
+        </is>
+      </c>
+      <c r="F760" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" t="n">
+        <v>762</v>
+      </c>
+      <c r="B761" t="inlineStr">
+        <is>
+          <t>11/10/2026 08:33</t>
+        </is>
+      </c>
+      <c r="C761" t="n">
+        <v>5024</v>
+      </c>
+      <c r="D761" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E761" t="inlineStr">
+        <is>
+          <t>Engenharia Organizacional</t>
+        </is>
+      </c>
+      <c r="F761" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="762">
+      <c r="A762" t="n">
+        <v>763</v>
+      </c>
+      <c r="B762" t="inlineStr">
+        <is>
+          <t>11/10/2026 08:34</t>
+        </is>
+      </c>
+      <c r="C762" t="inlineStr">
+        <is>
+          <t>2658</t>
+        </is>
+      </c>
+      <c r="D762" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E762" t="inlineStr">
+        <is>
+          <t>Gestão da Informação</t>
+        </is>
+      </c>
+      <c r="F762" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="763">
+      <c r="A763" t="n">
+        <v>764</v>
+      </c>
+      <c r="B763" t="inlineStr">
+        <is>
+          <t>11/10/2026 08:35</t>
+        </is>
+      </c>
+      <c r="C763" t="n">
+        <v>5452</v>
+      </c>
+      <c r="D763" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E763" t="inlineStr">
+        <is>
+          <t>Engenharia do Trabalho</t>
+        </is>
+      </c>
+      <c r="F763" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="764">
+      <c r="A764" t="n">
+        <v>765</v>
+      </c>
+      <c r="B764" t="inlineStr">
+        <is>
+          <t>11/10/2026 08:36</t>
+        </is>
+      </c>
+      <c r="C764" t="n">
+        <v>571</v>
+      </c>
+      <c r="D764" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E764" t="inlineStr">
+        <is>
+          <t>Gestão da Qualidade</t>
+        </is>
+      </c>
+      <c r="F764" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" t="n">
+        <v>766</v>
+      </c>
+      <c r="B765" t="inlineStr">
+        <is>
+          <t>11/10/2026 08:37</t>
+        </is>
+      </c>
+      <c r="C765" t="n">
+        <v>761</v>
+      </c>
+      <c r="D765" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E765" t="inlineStr">
+        <is>
+          <t>Engenharia Organizacional</t>
+        </is>
+      </c>
+      <c r="F765" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="766">
+      <c r="A766" t="n">
+        <v>767</v>
+      </c>
+      <c r="B766" t="inlineStr">
+        <is>
+          <t>11/10/2026 08:40</t>
+        </is>
+      </c>
+      <c r="C766" t="n">
+        <v>4943</v>
+      </c>
+      <c r="D766" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E766" t="inlineStr">
+        <is>
+          <t>Planejamento e Controle da Produção</t>
+        </is>
+      </c>
+      <c r="F766" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="767">
+      <c r="A767" t="n">
+        <v>768</v>
+      </c>
+      <c r="B767" t="inlineStr">
+        <is>
+          <t>11/10/2026 08:42</t>
+        </is>
+      </c>
+      <c r="C767" t="n">
+        <v>792</v>
+      </c>
+      <c r="D767" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E767" t="inlineStr">
+        <is>
+          <t>Gestão de Projetos</t>
+        </is>
+      </c>
+      <c r="F767" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" t="n">
+        <v>769</v>
+      </c>
+      <c r="B768" t="inlineStr">
+        <is>
+          <t>11/10/2026 08:46</t>
+        </is>
+      </c>
+      <c r="C768" t="n">
+        <v>5160</v>
+      </c>
+      <c r="D768" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E768" t="inlineStr">
+        <is>
+          <t>Gestão de Projetos</t>
+        </is>
+      </c>
+      <c r="F768" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="769">
+      <c r="A769" t="n">
+        <v>770</v>
+      </c>
+      <c r="B769" t="inlineStr">
+        <is>
+          <t>11/10/2026 08:48</t>
+        </is>
+      </c>
+      <c r="C769" t="n">
+        <v>829</v>
+      </c>
+      <c r="D769" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E769" t="inlineStr">
+        <is>
+          <t>Engenharia Organizacional</t>
+        </is>
+      </c>
+      <c r="F769" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" t="n">
+        <v>771</v>
+      </c>
+      <c r="B770" t="inlineStr">
+        <is>
+          <t>11/10/2026 08:49</t>
+        </is>
+      </c>
+      <c r="C770" t="n">
+        <v>5118</v>
+      </c>
+      <c r="D770" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E770" t="inlineStr">
+        <is>
+          <t>Gestão da Qualidade</t>
+        </is>
+      </c>
+      <c r="F770" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="771">
+      <c r="A771" t="n">
+        <v>772</v>
+      </c>
+      <c r="B771" t="inlineStr">
+        <is>
+          <t>11/10/2026 08:53</t>
+        </is>
+      </c>
+      <c r="C771" t="n">
+        <v>4980</v>
+      </c>
+      <c r="D771" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E771" t="inlineStr">
+        <is>
+          <t>Engenharia Organizacional</t>
+        </is>
+      </c>
+      <c r="F771" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="772">
+      <c r="A772" t="n">
+        <v>773</v>
+      </c>
+      <c r="B772" t="inlineStr">
+        <is>
+          <t>11/10/2026 08:55</t>
+        </is>
+      </c>
+      <c r="C772" t="n">
+        <v>5144</v>
+      </c>
+      <c r="D772" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E772" t="inlineStr">
+        <is>
+          <t>Gestão da Produção e Operações</t>
+        </is>
+      </c>
+      <c r="F772" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" t="n">
+        <v>774</v>
+      </c>
+      <c r="B773" t="inlineStr">
+        <is>
+          <t>11/10/2026 09:00</t>
+        </is>
+      </c>
+      <c r="C773" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D773" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E773" t="inlineStr">
+        <is>
+          <t>Engenharia Organizacional</t>
+        </is>
+      </c>
+      <c r="F773" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="774">
+      <c r="A774" t="n">
+        <v>775</v>
+      </c>
+      <c r="B774" t="inlineStr">
+        <is>
+          <t>11/10/2026 09:02</t>
+        </is>
+      </c>
+      <c r="C774" t="n">
+        <v>3314</v>
+      </c>
+      <c r="D774" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E774" t="inlineStr">
+        <is>
+          <t>Engenharia de Métodos e Processos</t>
+        </is>
+      </c>
+      <c r="F774" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" t="n">
+        <v>776</v>
+      </c>
+      <c r="B775" t="inlineStr">
+        <is>
+          <t>11/10/2026 09:02</t>
+        </is>
+      </c>
+      <c r="C775" t="n">
+        <v>5639</v>
+      </c>
+      <c r="D775" t="inlineStr">
+        <is>
+          <t>Conhecimentos Específicos</t>
+        </is>
+      </c>
+      <c r="E775" t="inlineStr">
+        <is>
+          <t>Gestão da Cadeia de Suprimentos</t>
+        </is>
+      </c>
+      <c r="F775" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="776">
+      <c r="A776" t="n">
+        <v>777</v>
+      </c>
+      <c r="B776" t="inlineStr">
+        <is>
+          <t>11/10/2026 09:09</t>
+        </is>
+      </c>
+      <c r="C776" t="inlineStr">
+        <is>
+          <t>5206</t>
+        </is>
+      </c>
+      <c r="D776" t="inlineStr">
+        <is>
+          <t>Contabilidade De Custos</t>
+        </is>
+      </c>
+      <c r="E776" t="inlineStr">
+        <is>
+          <t>Apuração Do Custo De Produção</t>
+        </is>
+      </c>
+      <c r="F776" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="777">
+      <c r="A777" t="n">
+        <v>778</v>
+      </c>
+      <c r="B777" t="inlineStr">
+        <is>
+          <t>11/10/2026 09:09</t>
+        </is>
+      </c>
+      <c r="C777" t="inlineStr">
+        <is>
+          <t>3199</t>
+        </is>
+      </c>
+      <c r="D777" t="inlineStr">
+        <is>
+          <t>Contabilidade Gerencial</t>
+        </is>
+      </c>
+      <c r="E777" t="inlineStr">
+        <is>
+          <t>Aspectos Introdutórios</t>
+        </is>
+      </c>
+      <c r="F777" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="778">
+      <c r="A778" t="n">
+        <v>779</v>
+      </c>
+      <c r="B778" t="inlineStr">
+        <is>
+          <t>11/10/2026 09:12</t>
+        </is>
+      </c>
+      <c r="C778" t="n">
+        <v>2559</v>
+      </c>
+      <c r="D778" t="inlineStr">
+        <is>
+          <t>Contratação</t>
+        </is>
+      </c>
+      <c r="E778" t="inlineStr">
+        <is>
+          <t>Lei nº 14.129 - 2021</t>
+        </is>
+      </c>
+      <c r="F778" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" t="n">
+        <v>780</v>
+      </c>
+      <c r="B779" t="inlineStr">
+        <is>
+          <t>11/10/2026 09:13</t>
+        </is>
+      </c>
+      <c r="C779" t="n">
+        <v>4829</v>
+      </c>
+      <c r="D779" t="inlineStr">
+        <is>
+          <t>Contratação</t>
+        </is>
+      </c>
+      <c r="E779" t="inlineStr">
+        <is>
+          <t>Lei Complementar Nº 123 - 2006 e Lei Complementar Nº 155 - 2016</t>
+        </is>
+      </c>
+      <c r="F779" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" t="n">
+        <v>781</v>
+      </c>
+      <c r="B780" t="inlineStr">
+        <is>
+          <t>11/10/2026 09:14</t>
+        </is>
+      </c>
+      <c r="C780" t="n">
+        <v>4867</v>
+      </c>
+      <c r="D780" t="inlineStr">
+        <is>
+          <t>Contratação</t>
+        </is>
+      </c>
+      <c r="E780" t="inlineStr">
+        <is>
+          <t>Lei Complementar Nº 123 - 2006 e Lei Complementar Nº 155 - 2016</t>
+        </is>
+      </c>
+      <c r="F780" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" t="n">
+        <v>782</v>
+      </c>
+      <c r="B781" t="inlineStr">
+        <is>
+          <t>11/10/2026 09:16</t>
+        </is>
+      </c>
+      <c r="C781" t="inlineStr">
+        <is>
+          <t>2537</t>
+        </is>
+      </c>
+      <c r="D781" t="inlineStr">
+        <is>
+          <t>Contratação</t>
+        </is>
+      </c>
+      <c r="E781" t="inlineStr">
+        <is>
+          <t>Lei nº 14.129 - 2021</t>
+        </is>
+      </c>
+      <c r="F781" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="782">
+      <c r="A782" t="n">
+        <v>783</v>
+      </c>
+      <c r="B782" t="inlineStr">
+        <is>
+          <t>11/10/2026 09:20</t>
+        </is>
+      </c>
+      <c r="C782" t="n">
+        <v>4849</v>
+      </c>
+      <c r="D782" t="inlineStr">
+        <is>
+          <t>Contratação</t>
+        </is>
+      </c>
+      <c r="E782" t="inlineStr">
+        <is>
+          <t>Lei nº 14.129 - 2021</t>
+        </is>
+      </c>
+      <c r="F782" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" t="n">
+        <v>784</v>
+      </c>
+      <c r="B783" t="inlineStr">
+        <is>
+          <t>11/10/2026 09:24</t>
+        </is>
+      </c>
+      <c r="C783" t="n">
+        <v>2592</v>
+      </c>
+      <c r="D783" t="inlineStr">
+        <is>
+          <t>Estatística</t>
+        </is>
+      </c>
+      <c r="E783" t="inlineStr">
+        <is>
+          <t>Análise Combinatória</t>
+        </is>
+      </c>
+      <c r="F783" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" t="n">
+        <v>785</v>
+      </c>
+      <c r="B784" t="inlineStr">
+        <is>
+          <t>11/10/2026 09:37</t>
+        </is>
+      </c>
+      <c r="C784" t="n">
+        <v>881</v>
+      </c>
+      <c r="D784" t="inlineStr">
+        <is>
+          <t>Inglês</t>
+        </is>
+      </c>
+      <c r="E784" t="inlineStr">
+        <is>
+          <t>Vocabulary &amp; Semantics</t>
+        </is>
+      </c>
+      <c r="F784" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" t="n">
+        <v>786</v>
+      </c>
+      <c r="B785" t="inlineStr">
+        <is>
+          <t>11/10/2026 09:37</t>
+        </is>
+      </c>
+      <c r="C785" t="n">
+        <v>880</v>
+      </c>
+      <c r="D785" t="inlineStr">
+        <is>
+          <t>Inglês</t>
+        </is>
+      </c>
+      <c r="E785" t="inlineStr">
+        <is>
+          <t>Vocabulary &amp; Semantics</t>
+        </is>
+      </c>
+      <c r="F785" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="786">
+      <c r="A786" t="n">
+        <v>787</v>
+      </c>
+      <c r="B786" t="inlineStr">
+        <is>
+          <t>11/10/2026 09:38</t>
+        </is>
+      </c>
+      <c r="C786" t="n">
+        <v>879</v>
+      </c>
+      <c r="D786" t="inlineStr">
+        <is>
+          <t>Inglês</t>
+        </is>
+      </c>
+      <c r="E786" t="inlineStr">
+        <is>
+          <t>Reading Comprehension</t>
+        </is>
+      </c>
+      <c r="F786" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" t="n">
+        <v>788</v>
+      </c>
+      <c r="B787" t="inlineStr">
+        <is>
+          <t>11/10/2026 09:39</t>
+        </is>
+      </c>
+      <c r="C787" t="n">
+        <v>878</v>
+      </c>
+      <c r="D787" t="inlineStr">
+        <is>
+          <t>Inglês</t>
+        </is>
+      </c>
+      <c r="E787" t="inlineStr">
+        <is>
+          <t>Reading Comprehension</t>
+        </is>
+      </c>
+      <c r="F787" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" t="n">
+        <v>789</v>
+      </c>
+      <c r="B788" t="inlineStr">
+        <is>
+          <t>11/10/2026 09:50</t>
+        </is>
+      </c>
+      <c r="C788" t="n">
+        <v>950</v>
+      </c>
+      <c r="D788" t="inlineStr">
+        <is>
+          <t>Inglês</t>
+        </is>
+      </c>
+      <c r="E788" t="inlineStr">
+        <is>
+          <t>Vocabulary &amp; Semantics</t>
+        </is>
+      </c>
+      <c r="F788" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" t="n">
+        <v>790</v>
+      </c>
+      <c r="B789" t="inlineStr">
+        <is>
+          <t>11/10/2026 10:01</t>
+        </is>
+      </c>
+      <c r="C789" t="n">
+        <v>1268</v>
+      </c>
+      <c r="D789" t="inlineStr">
+        <is>
+          <t>Matemática Financeira</t>
+        </is>
+      </c>
+      <c r="E789" t="inlineStr">
+        <is>
+          <t>Juros Compostos</t>
+        </is>
+      </c>
+      <c r="F789" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" t="n">
+        <v>791</v>
+      </c>
+      <c r="B790" t="inlineStr">
+        <is>
+          <t>11/10/2026 10:02</t>
+        </is>
+      </c>
+      <c r="C790" t="n">
+        <v>3122</v>
+      </c>
+      <c r="D790" t="inlineStr">
+        <is>
+          <t>Matemática Financeira</t>
+        </is>
+      </c>
+      <c r="E790" t="inlineStr">
+        <is>
+          <t>Equivalência de Capitais</t>
+        </is>
+      </c>
+      <c r="F790" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" t="n">
+        <v>792</v>
+      </c>
+      <c r="B791" t="inlineStr">
+        <is>
+          <t>11/10/2026 10:04</t>
+        </is>
+      </c>
+      <c r="C791" t="n">
+        <v>3304</v>
+      </c>
+      <c r="D791" t="inlineStr">
+        <is>
+          <t>Matemática Financeira</t>
+        </is>
+      </c>
+      <c r="E791" t="inlineStr">
+        <is>
+          <t>Análise de Investimentos</t>
+        </is>
+      </c>
+      <c r="F791" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" t="n">
+        <v>793</v>
+      </c>
+      <c r="B792" t="inlineStr">
+        <is>
+          <t>11/10/2026 10:10</t>
+        </is>
+      </c>
+      <c r="C792" t="n">
+        <v>3429</v>
+      </c>
+      <c r="D792" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="E792" t="inlineStr">
+        <is>
+          <t>Semântica</t>
+        </is>
+      </c>
+      <c r="F792" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" t="n">
+        <v>794</v>
+      </c>
+      <c r="B793" t="inlineStr">
+        <is>
+          <t>11/10/2026 10:10</t>
+        </is>
+      </c>
+      <c r="C793" t="inlineStr">
+        <is>
+          <t>3430</t>
+        </is>
+      </c>
+      <c r="D793" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="E793" t="inlineStr">
+        <is>
+          <t>Morfologia</t>
+        </is>
+      </c>
+      <c r="F793" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="794">
+      <c r="A794" t="n">
+        <v>795</v>
+      </c>
+      <c r="B794" t="inlineStr">
+        <is>
+          <t>11/10/2026 10:12</t>
+        </is>
+      </c>
+      <c r="C794" t="n">
+        <v>3428</v>
+      </c>
+      <c r="D794" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="E794" t="inlineStr">
+        <is>
+          <t>Compreensão e Interpretação de Textos</t>
+        </is>
+      </c>
+      <c r="F794" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" t="n">
+        <v>796</v>
+      </c>
+      <c r="B795" t="inlineStr">
+        <is>
+          <t>11/10/2026 10:13</t>
+        </is>
+      </c>
+      <c r="C795" t="n">
+        <v>3427</v>
+      </c>
+      <c r="D795" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="E795" t="inlineStr">
+        <is>
+          <t>Compreensão e Interpretação de Textos</t>
+        </is>
+      </c>
+      <c r="F795" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" t="n">
+        <v>797</v>
+      </c>
+      <c r="B796" t="inlineStr">
+        <is>
+          <t>11/10/2026 10:14</t>
+        </is>
+      </c>
+      <c r="C796" t="n">
+        <v>3426</v>
+      </c>
+      <c r="D796" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="E796" t="inlineStr">
+        <is>
+          <t>Regência Verbal e Nominal; e Crase</t>
+        </is>
+      </c>
+      <c r="F796" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" t="n">
+        <v>798</v>
+      </c>
+      <c r="B797" t="inlineStr">
+        <is>
+          <t>11/10/2026 10:15</t>
+        </is>
+      </c>
+      <c r="C797" t="n">
+        <v>3425</v>
+      </c>
+      <c r="D797" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="E797" t="inlineStr">
+        <is>
+          <t>Mecanismos de Coesão Textual</t>
+        </is>
+      </c>
+      <c r="F797" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" t="n">
+        <v>799</v>
+      </c>
+      <c r="B798" t="inlineStr">
+        <is>
+          <t>11/10/2026 10:22</t>
+        </is>
+      </c>
+      <c r="C798" t="n">
+        <v>3424</v>
+      </c>
+      <c r="D798" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="E798" t="inlineStr">
+        <is>
+          <t>Relações de Coordenação entre Orações e entre Termos da Oração</t>
+        </is>
+      </c>
+      <c r="F798" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" t="n">
+        <v>800</v>
+      </c>
+      <c r="B799" t="inlineStr">
+        <is>
+          <t>11/10/2026 10:24</t>
+        </is>
+      </c>
+      <c r="C799" t="n">
+        <v>6200</v>
+      </c>
+      <c r="D799" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="E799" t="inlineStr">
+        <is>
+          <t>Compreensão e Interpretação de Textos</t>
+        </is>
+      </c>
+      <c r="F799" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" t="n">
+        <v>801</v>
+      </c>
+      <c r="B800" t="inlineStr">
+        <is>
+          <t>11/10/2026 10:35</t>
+        </is>
+      </c>
+      <c r="C800" t="n">
+        <v>6171</v>
+      </c>
+      <c r="D800" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="E800" t="inlineStr">
+        <is>
+          <t>Compreensão e Interpretação de Textos</t>
+        </is>
+      </c>
+      <c r="F800" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" t="n">
+        <v>802</v>
+      </c>
+      <c r="B801" t="inlineStr">
+        <is>
+          <t>11/10/2026 10:35</t>
+        </is>
+      </c>
+      <c r="C801" t="n">
+        <v>6170</v>
+      </c>
+      <c r="D801" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="E801" t="inlineStr">
+        <is>
+          <t>Compreensão e Interpretação de Textos</t>
+        </is>
+      </c>
+      <c r="F801" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" t="n">
+        <v>803</v>
+      </c>
+      <c r="B802" t="inlineStr">
+        <is>
+          <t>11/10/2026 10:36</t>
+        </is>
+      </c>
+      <c r="C802" t="n">
+        <v>6169</v>
+      </c>
+      <c r="D802" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="E802" t="inlineStr">
+        <is>
+          <t>Compreensão e Interpretação de Textos</t>
+        </is>
+      </c>
+      <c r="F802" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" t="n">
+        <v>804</v>
+      </c>
+      <c r="B803" t="inlineStr">
+        <is>
+          <t>11/10/2026 10:36</t>
+        </is>
+      </c>
+      <c r="C803" t="n">
+        <v>6168</v>
+      </c>
+      <c r="D803" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="E803" t="inlineStr">
+        <is>
+          <t>Compreensão e Interpretação de Textos</t>
+        </is>
+      </c>
+      <c r="F803" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" t="n">
+        <v>805</v>
+      </c>
+      <c r="B804" t="inlineStr">
+        <is>
+          <t>11/10/2026 10:37</t>
+        </is>
+      </c>
+      <c r="C804" t="n">
+        <v>6167</v>
+      </c>
+      <c r="D804" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="E804" t="inlineStr">
+        <is>
+          <t>Compreensão e Interpretação de Textos</t>
+        </is>
+      </c>
+      <c r="F804" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" t="n">
+        <v>806</v>
+      </c>
+      <c r="B805" t="inlineStr">
+        <is>
+          <t>11/10/2026 10:37</t>
+        </is>
+      </c>
+      <c r="C805" t="n">
+        <v>6166</v>
+      </c>
+      <c r="D805" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="E805" t="inlineStr">
+        <is>
+          <t>Mecanismos de Coesão Textual</t>
+        </is>
+      </c>
+      <c r="F805" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" t="n">
+        <v>807</v>
+      </c>
+      <c r="B806" t="inlineStr">
+        <is>
+          <t>11/10/2026 10:38</t>
+        </is>
+      </c>
+      <c r="C806" t="n">
+        <v>6098</v>
+      </c>
+      <c r="D806" t="inlineStr">
+        <is>
+          <t>Português</t>
+        </is>
+      </c>
+      <c r="E806" t="inlineStr">
+        <is>
+          <t>Relações de Coordenação entre Orações e entre Termos da Oração</t>
+        </is>
+      </c>
+      <c r="F806" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:F720"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>